<commit_message>
Fix review findings in the DbLib and Altium 365 exporters
Map full designator prefixes (LED, IC, CN, JP), stop part-number
collisions and value-less parts from dropping rows, point Library Path
at the per-symbol SchLib files, close the SQLite connection, surface
payload errors from parameter updates, dedupe plan items, and exit
non-zero when any part fails to push. Adds tests/test_review_altium.py.
</commit_message>
<xml_diff>
--- a/out/altium/parts.xlsx
+++ b/out/altium/parts.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="137">
   <si>
     <t>Part Number</t>
   </si>
@@ -82,7 +82,7 @@
     <t>Capacitor</t>
   </si>
   <si>
-    <t>SchLib\Capacitors.SchLib</t>
+    <t>SchLib\Capacitor.SchLib</t>
   </si>
   <si>
     <t>C_0402_1005Metric</t>
@@ -127,7 +127,13 @@
     <t>FTSH-105-01-L-DV-K</t>
   </si>
   <si>
-    <t>SchLib\Connectors.SchLib</t>
+    <t>SchLib\TYPE-C-31-M-12.SchLib</t>
+  </si>
+  <si>
+    <t>SchLib\SM04B-SRSS-TB(LF)(SN).SchLib</t>
+  </si>
+  <si>
+    <t>SchLib\FTSH-105-01-L-DV-K.SchLib</t>
   </si>
   <si>
     <t>USB_C_Receptacle_16P</t>
@@ -187,7 +193,7 @@
     <t>X322512MSB4SI</t>
   </si>
   <si>
-    <t>SchLib\Crystals.SchLib</t>
+    <t>SchLib\X322512MSB4SI.SchLib</t>
   </si>
   <si>
     <t>Crystal_SMD_3225-4Pin</t>
@@ -214,7 +220,7 @@
     <t>KT-0603R</t>
   </si>
   <si>
-    <t>SchLib\Diodes.SchLib</t>
+    <t>SchLib\KT-0603R.SchLib</t>
   </si>
   <si>
     <t>LED_0603_1608Metric</t>
@@ -256,7 +262,22 @@
     <t>TPS62162DSGR</t>
   </si>
   <si>
-    <t>SchLib\ICs.SchLib</t>
+    <t>SchLib\STM32F103C8T6.SchLib</t>
+  </si>
+  <si>
+    <t>SchLib\AMS1117-3.3.SchLib</t>
+  </si>
+  <si>
+    <t>SchLib\ESP32-S3-WROOM-1-N16R8.SchLib</t>
+  </si>
+  <si>
+    <t>SchLib\TPS62133RGTR.SchLib</t>
+  </si>
+  <si>
+    <t>SchLib\CH340C.SchLib</t>
+  </si>
+  <si>
+    <t>SchLib\TPS62162DSGR.SchLib</t>
   </si>
   <si>
     <t>LQFP-48_7x7mm_P0.5mm</t>
@@ -361,7 +382,7 @@
     <t>Resistor</t>
   </si>
   <si>
-    <t>SchLib\Resistors.SchLib</t>
+    <t>SchLib\Resistor.SchLib</t>
   </si>
   <si>
     <t>R_0603_1608Metric</t>
@@ -391,7 +412,7 @@
     <t>AO3401A</t>
   </si>
   <si>
-    <t>SchLib\Transistors.SchLib</t>
+    <t>SchLib\AO3401A.SchLib</t>
   </si>
   <si>
     <t>SOT-23</t>
@@ -945,22 +966,22 @@
         <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
         <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H2" t="s">
         <v>32</v>
       </c>
       <c r="I2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J2" t="s">
         <v>32</v>
@@ -969,19 +990,19 @@
         <v>27</v>
       </c>
       <c r="L2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="O2" t="s">
         <v>27</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="Q2" t="s">
         <v>30</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -992,25 +1013,25 @@
         <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E3" t="s">
         <v>22</v>
       </c>
       <c r="F3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H3" t="s">
         <v>33</v>
       </c>
       <c r="I3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="J3" t="s">
         <v>33</v>
@@ -1019,19 +1040,19 @@
         <v>27</v>
       </c>
       <c r="L3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="O3" t="s">
         <v>27</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="Q3" t="s">
         <v>30</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -1042,25 +1063,25 @@
         <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E4" t="s">
         <v>22</v>
       </c>
       <c r="F4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H4" t="s">
         <v>34</v>
       </c>
       <c r="I4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J4" t="s">
         <v>34</v>
@@ -1140,52 +1161,52 @@
     </row>
     <row r="2" spans="1:18">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E2" t="s">
         <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="J2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="K2" t="s">
         <v>27</v>
       </c>
       <c r="L2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O2" t="s">
         <v>27</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="Q2" t="s">
         <v>30</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1260,52 +1281,52 @@
     </row>
     <row r="2" spans="1:18">
       <c r="A2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E2" t="s">
         <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="I2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K2" t="s">
         <v>27</v>
       </c>
       <c r="L2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="O2" t="s">
         <v>27</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="Q2" t="s">
         <v>30</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1380,284 +1401,284 @@
     </row>
     <row r="2" spans="1:18">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D2" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="E2" t="s">
         <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="G2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I2" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="J2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K2" t="s">
         <v>27</v>
       </c>
       <c r="L2" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="O2" t="s">
         <v>27</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="Q2" t="s">
         <v>30</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:18">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="E3" t="s">
         <v>22</v>
       </c>
       <c r="F3" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="G3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I3" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="J3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K3" t="s">
         <v>27</v>
       </c>
       <c r="L3" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="O3" t="s">
         <v>27</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="Q3" t="s">
         <v>30</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:18">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C4" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D4" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="E4" t="s">
         <v>22</v>
       </c>
       <c r="F4" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="G4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I4" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="J4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K4" t="s">
         <v>27</v>
       </c>
       <c r="L4" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="O4" t="s">
         <v>27</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="Q4" t="s">
         <v>30</v>
       </c>
       <c r="R4" s="1" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:18">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D5" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="E5" t="s">
         <v>22</v>
       </c>
       <c r="F5" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="G5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I5" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="J5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K5" t="s">
         <v>27</v>
       </c>
       <c r="L5" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="O5" t="s">
         <v>27</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="Q5" t="s">
         <v>30</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:18">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D6" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="E6" t="s">
         <v>22</v>
       </c>
       <c r="F6" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="G6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I6" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="J6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="K6" t="s">
         <v>27</v>
       </c>
       <c r="L6" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="O6" t="s">
         <v>27</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="Q6" t="s">
         <v>30</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:18">
       <c r="A7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C7" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="D7" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="E7" t="s">
         <v>22</v>
       </c>
       <c r="F7" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="G7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I7" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="J7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1740,53 +1761,53 @@
     </row>
     <row r="2" spans="1:18">
       <c r="A2" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="B2" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="C2" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="D2" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="E2" t="s">
         <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="G2" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="H2">
         <f>Value</f>
         <v>0</v>
       </c>
       <c r="I2" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="J2" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="K2" t="s">
         <v>27</v>
       </c>
       <c r="L2" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="O2" t="s">
         <v>27</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="Q2" t="s">
         <v>30</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -1861,52 +1882,52 @@
     </row>
     <row r="2" spans="1:18">
       <c r="A2" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B2" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="C2" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="D2" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="E2" t="s">
         <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="G2" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="H2" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="I2" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="J2" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="K2" t="s">
         <v>27</v>
       </c>
       <c r="L2" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="O2" t="s">
         <v>27</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="Q2" t="s">
         <v>30</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>